<commit_message>
Added logistic regression intro lecture
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD07EB4-E65F-4874-B597-5A3ED3A29C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EB92B0-7495-4129-91CB-A7B68B56CEAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="187">
   <si>
     <t>week</t>
   </si>
@@ -132,18 +132,9 @@
     <t>Exam 01</t>
   </si>
   <si>
-    <t>MLR: Inference, conditions, variable transformations</t>
-  </si>
-  <si>
-    <t>/slides/15-mlr-inference.html</t>
-  </si>
-  <si>
     <t>/hw/hw-03.html</t>
   </si>
   <si>
-    <t>HW 03 assigned</t>
-  </si>
-  <si>
     <t>Lab: Project proposal</t>
   </si>
   <si>
@@ -592,6 +583,18 @@
   </si>
   <si>
     <t>/ae/ae-17-multicollinearity.html</t>
+  </si>
+  <si>
+    <t>/prepare/logistic-regression-prep.html</t>
+  </si>
+  <si>
+    <t>/slides/24-logistic-intro.html</t>
+  </si>
+  <si>
+    <t>/ae/ae-18-logistic-intro.html</t>
+  </si>
+  <si>
+    <t>Logistic regression intro continued</t>
   </si>
 </sst>
 </file>
@@ -976,7 +979,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -1125,9 +1128,6 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1481,7 +1481,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="16.5">
       <c r="A1" s="17" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1519,7 +1519,7 @@
     </row>
     <row r="2" spans="1:12" ht="49.5">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
@@ -1538,17 +1538,17 @@
         <v>13</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
       <c r="L2" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="33">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="5" t="s">
@@ -1561,7 +1561,7 @@
         <v>16</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
@@ -1570,12 +1570,12 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="L3" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="66">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B4" s="4">
         <v>2</v>
@@ -1587,10 +1587,10 @@
         <v>45530</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="5" spans="1:12" ht="66">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="5" t="s">
@@ -1615,7 +1615,7 @@
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>22</v>
@@ -1633,7 +1633,7 @@
     </row>
     <row r="6" spans="1:12" ht="49.5">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="5" t="s">
@@ -1643,14 +1643,14 @@
         <v>45534</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -1659,7 +1659,7 @@
     </row>
     <row r="7" spans="1:12" ht="16.5">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B7" s="4">
         <v>3</v>
@@ -1671,12 +1671,12 @@
         <v>45537</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="99">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5" t="s">
@@ -1689,26 +1689,26 @@
         <v>23</v>
       </c>
       <c r="F8" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>107</v>
-      </c>
       <c r="H8" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>29</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="L8" s="8"/>
     </row>
     <row r="9" spans="1:12" ht="165">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="5" t="s">
@@ -1718,21 +1718,21 @@
         <v>45541</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="8"/>
       <c r="K9" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>26</v>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="10" spans="1:12" ht="115.5">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B10" s="4">
         <v>4</v>
@@ -1755,10 +1755,10 @@
         <v>27</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="8"/>
@@ -1768,7 +1768,7 @@
     </row>
     <row r="11" spans="1:12" ht="148.5">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="5" t="s">
@@ -1778,14 +1778,14 @@
         <v>45546</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="5"/>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="12" spans="1:12" ht="66">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="5" t="s">
@@ -1806,26 +1806,26 @@
         <v>28</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L12" s="8"/>
     </row>
     <row r="13" spans="1:12" ht="99">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B13" s="32">
         <v>5</v>
@@ -1837,16 +1837,16 @@
         <v>45551</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I13" s="37"/>
       <c r="J13" s="35"/>
@@ -1855,7 +1855,7 @@
     </row>
     <row r="14" spans="1:12" ht="66">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="33" t="s">
@@ -1865,16 +1865,16 @@
         <v>45553</v>
       </c>
       <c r="E14" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>121</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="35"/>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="15" spans="1:12" ht="49.5">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B15" s="32"/>
       <c r="C15" s="33" t="s">
@@ -1893,29 +1893,29 @@
         <v>45555</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I15" s="37" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J15" s="35"/>
       <c r="K15" s="36" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="L15" s="35"/>
     </row>
     <row r="16" spans="1:12" ht="49.5">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B16" s="32">
         <v>6</v>
@@ -1927,25 +1927,25 @@
         <v>45558</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G16" s="36"/>
       <c r="H16" s="39"/>
       <c r="I16" s="37"/>
       <c r="J16" s="41" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="L16" s="35"/>
     </row>
     <row r="17" spans="1:12" ht="99">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="33" t="s">
@@ -1955,7 +1955,7 @@
         <v>45560</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="35"/>
@@ -1964,7 +1964,7 @@
     </row>
     <row r="18" spans="1:12" ht="33">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="33" t="s">
@@ -1974,29 +1974,29 @@
         <v>45562</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="G18" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="39" t="s">
         <v>132</v>
       </c>
-      <c r="H18" s="39" t="s">
-        <v>135</v>
-      </c>
       <c r="I18" s="37" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J18" s="35"/>
       <c r="K18" s="24" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="L18" s="35"/>
     </row>
     <row r="19" spans="1:12" ht="66">
       <c r="A19" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B19" s="4">
         <v>7</v>
@@ -2008,16 +2008,16 @@
         <v>45565</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F19" s="45" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I19" s="24"/>
       <c r="J19" s="24"/>
@@ -2025,7 +2025,7 @@
     </row>
     <row r="20" spans="1:12" ht="66">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="43" t="s">
@@ -2035,16 +2035,16 @@
         <v>45567</v>
       </c>
       <c r="E20" s="40" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F20" s="45" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
@@ -2053,7 +2053,7 @@
     </row>
     <row r="21" spans="1:12" ht="49.5">
       <c r="A21" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="42" t="s">
@@ -2063,29 +2063,29 @@
         <v>45569</v>
       </c>
       <c r="E21" s="44" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F21" s="46" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G21" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="I21" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>151</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="8" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="L21" s="8"/>
     </row>
     <row r="22" spans="1:12" ht="66">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B22" s="4">
         <v>8</v>
@@ -2097,16 +2097,16 @@
         <v>45572</v>
       </c>
       <c r="E22" s="44" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F22" s="46" t="s">
+        <v>153</v>
+      </c>
+      <c r="G22" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="H22" s="27" t="s">
         <v>156</v>
-      </c>
-      <c r="G22" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>159</v>
       </c>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
@@ -2115,7 +2115,7 @@
     </row>
     <row r="23" spans="1:12" ht="33">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="5" t="s">
@@ -2128,13 +2128,13 @@
         <v>30</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
@@ -2143,7 +2143,7 @@
     </row>
     <row r="24" spans="1:12" ht="16.5">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="5" t="s">
@@ -2161,13 +2161,13 @@
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="L24" s="8"/>
     </row>
     <row r="25" spans="1:12" ht="66">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B25" s="4">
         <v>9</v>
@@ -2179,7 +2179,7 @@
         <v>45579</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -2187,13 +2187,13 @@
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="L25" s="8"/>
     </row>
     <row r="26" spans="1:12" ht="66">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="9" t="s">
@@ -2203,7 +2203,7 @@
         <v>45581</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -2215,7 +2215,7 @@
     </row>
     <row r="27" spans="1:12" ht="66">
       <c r="A27" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="5" t="s">
@@ -2225,7 +2225,7 @@
         <v>45583</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
@@ -2237,7 +2237,7 @@
     </row>
     <row r="28" spans="1:12" ht="49.5">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B28" s="4">
         <v>10</v>
@@ -2249,16 +2249,16 @@
         <v>45586</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I28" s="13"/>
       <c r="J28" s="8"/>
@@ -2267,7 +2267,7 @@
     </row>
     <row r="29" spans="1:12" ht="66">
       <c r="A29" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="9" t="s">
@@ -2277,27 +2277,27 @@
         <v>45588</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>168</v>
-      </c>
       <c r="G29" s="26" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
       <c r="L29" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="99">
       <c r="A30" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="5" t="s">
@@ -2307,27 +2307,27 @@
         <v>45590</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="26" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="L30" s="8"/>
     </row>
     <row r="31" spans="1:12" ht="49.5">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B31" s="4">
         <v>11</v>
@@ -2339,16 +2339,16 @@
         <v>45593</v>
       </c>
       <c r="E31" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G31" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>178</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>181</v>
       </c>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
@@ -2357,7 +2357,7 @@
     </row>
     <row r="32" spans="1:12" ht="49.5">
       <c r="A32" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="9" t="s">
@@ -2367,29 +2367,29 @@
         <v>45595</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F32" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G32" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="G32" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>185</v>
-      </c>
       <c r="I32" s="49"/>
-      <c r="J32" s="53" t="s">
-        <v>174</v>
+      <c r="J32" s="52" t="s">
+        <v>171</v>
       </c>
       <c r="K32" s="49" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="L32" s="49"/>
     </row>
     <row r="33" spans="1:12" ht="49.5">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="5" t="s">
@@ -2399,40 +2399,47 @@
         <v>45597</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" s="8"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="53"/>
-      <c r="K33" s="53" t="s">
-        <v>173</v>
-      </c>
-      <c r="L33" s="53"/>
-    </row>
-    <row r="34" spans="1:12" ht="132">
-      <c r="B34" s="10"/>
+        <v>35</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G33" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I33" s="52"/>
+      <c r="K33" s="52" t="s">
+        <v>170</v>
+      </c>
+      <c r="L33" s="52"/>
+    </row>
+    <row r="34" spans="1:12" ht="82.5">
+      <c r="A34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="4">
+        <v>12</v>
+      </c>
       <c r="C34" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D34" s="6">
-        <v>45590</v>
+        <v>45600</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F34" s="8"/>
-      <c r="G34" s="9" t="s">
-        <v>33</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G34" s="9"/>
       <c r="H34" s="50"/>
-      <c r="I34" s="51" t="s">
-        <v>34</v>
-      </c>
+      <c r="I34" s="51"/>
       <c r="J34" s="50"/>
-      <c r="K34" s="51" t="s">
-        <v>35</v>
-      </c>
+      <c r="K34" s="51"/>
       <c r="L34" s="50"/>
     </row>
     <row r="35" spans="1:12" ht="49.5">
@@ -2442,14 +2449,14 @@
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
       <c r="I35" s="8"/>
       <c r="J35" s="9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K35" s="13"/>
       <c r="L35" s="8"/>
@@ -2465,14 +2472,14 @@
         <v>45595</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F36" s="8"/>
       <c r="G36" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I36" s="8"/>
       <c r="J36" s="8"/>
@@ -2488,19 +2495,19 @@
         <v>45597</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F37" s="8"/>
       <c r="G37" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I37" s="8"/>
       <c r="J37" s="8"/>
       <c r="K37" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L37" s="8"/>
     </row>
@@ -2513,7 +2520,7 @@
         <v>45598</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
@@ -2534,11 +2541,11 @@
         <v>45602</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F39" s="8"/>
       <c r="G39" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H39" s="13"/>
       <c r="I39" s="8"/>
@@ -2555,21 +2562,21 @@
         <v>45604</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F40" s="8"/>
       <c r="G40" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J40" s="8"/>
       <c r="K40" s="9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L40" s="8"/>
     </row>
@@ -2580,7 +2587,7 @@
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
@@ -2589,7 +2596,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="82.5">
@@ -2603,14 +2610,14 @@
         <v>45609</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F42" s="8"/>
       <c r="G42" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>
@@ -2626,30 +2633,30 @@
         <v>45611</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I43" s="13"/>
       <c r="J43" s="8"/>
       <c r="K43" s="15" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L43" s="8"/>
     </row>
     <row r="44" spans="1:12" ht="82.5">
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -2658,7 +2665,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="13"/>
       <c r="L44" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="33">
@@ -2672,17 +2679,17 @@
         <v>45616</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J45" s="8"/>
       <c r="K45" s="9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L45" s="8"/>
     </row>
@@ -2695,7 +2702,7 @@
         <v>45618</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -2712,7 +2719,7 @@
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -2733,20 +2740,20 @@
         <v>45623</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H48" s="13"/>
       <c r="I48" s="8"/>
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
       <c r="L48" s="5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="33">
@@ -2758,19 +2765,19 @@
         <v>45625</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I49" s="13"/>
       <c r="J49" s="8"/>
       <c r="K49" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L49" s="8"/>
     </row>
@@ -2781,7 +2788,7 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
@@ -2794,20 +2801,20 @@
     <row r="51" spans="2:12" ht="82.5">
       <c r="B51" s="10"/>
       <c r="C51" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D51" s="6">
         <v>45627</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="8"/>
       <c r="J51" s="9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="K51" s="13"/>
       <c r="L51" s="8"/>
@@ -2823,7 +2830,7 @@
         <v>45630</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
@@ -2842,7 +2849,7 @@
         <v>45632</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
@@ -2851,7 +2858,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
       <c r="L53" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="2:12" ht="66">
@@ -2861,39 +2868,39 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
       <c r="J54" s="16" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="K54" s="13"/>
       <c r="L54" s="8"/>
     </row>
     <row r="55" spans="2:12" ht="115.5">
       <c r="B55" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C55" s="8"/>
       <c r="D55" s="6">
         <v>45639</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
       <c r="J55" s="16" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="K55" s="8"/>
       <c r="L55" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding second logistic lecture
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{3C03FE42-C03A-49A6-A451-567437698B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3103AFE-DEDC-49E2-9C76-C986E4138A8C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF908AE-E5CA-4E1A-B547-FD183213F8E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="190">
   <si>
     <t>week</t>
   </si>
@@ -598,13 +598,19 @@
   </si>
   <si>
     <t>Logistic regression Prediction + Classification</t>
+  </si>
+  <si>
+    <t>/slides/25-logistic-intro2.html</t>
+  </si>
+  <si>
+    <t>/ae/ae-19-logistic-intro2.html</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1475,12 +1481,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C666FC1-734D-4F31-9D28-5509B94BC597}">
   <dimension ref="A1:L55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="16.5">
       <c r="A1" s="17" t="s">
         <v>84</v>
       </c>
@@ -1518,7 +1524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="49.5">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -1547,7 +1553,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="33">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1574,7 +1580,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="66">
       <c r="A4" t="s">
         <v>85</v>
       </c>
@@ -1598,7 +1604,7 @@
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
     </row>
-    <row r="5" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="66">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -1632,7 +1638,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="49.5">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1658,7 +1664,7 @@
       <c r="K6" s="28"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16.5">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -1675,7 +1681,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="99">
       <c r="A8" t="s">
         <v>85</v>
       </c>
@@ -1707,7 +1713,7 @@
       </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="181.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="165">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -1739,7 +1745,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="115.5">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -1767,7 +1773,7 @@
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="148.5">
       <c r="A11" t="s">
         <v>85</v>
       </c>
@@ -1792,7 +1798,7 @@
       <c r="K11" s="5"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="66">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -1824,7 +1830,7 @@
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="99">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1854,7 +1860,7 @@
       <c r="K13" s="36"/>
       <c r="L13" s="35"/>
     </row>
-    <row r="14" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="66">
       <c r="A14" t="s">
         <v>85</v>
       </c>
@@ -1882,7 +1888,7 @@
       <c r="K14" s="36"/>
       <c r="L14" s="35"/>
     </row>
-    <row r="15" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="49.5">
       <c r="A15" t="s">
         <v>85</v>
       </c>
@@ -1914,7 +1920,7 @@
       </c>
       <c r="L15" s="35"/>
     </row>
-    <row r="16" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="49.5">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -1944,7 +1950,7 @@
       </c>
       <c r="L16" s="35"/>
     </row>
-    <row r="17" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="99">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -1963,7 +1969,7 @@
       <c r="K17" s="36"/>
       <c r="L17" s="35"/>
     </row>
-    <row r="18" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="33">
       <c r="A18" t="s">
         <v>85</v>
       </c>
@@ -1995,7 +2001,7 @@
       </c>
       <c r="L18" s="35"/>
     </row>
-    <row r="19" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="66">
       <c r="A19" t="s">
         <v>85</v>
       </c>
@@ -2024,7 +2030,7 @@
       <c r="J19" s="24"/>
       <c r="L19" s="24"/>
     </row>
-    <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="66">
       <c r="A20" t="s">
         <v>85</v>
       </c>
@@ -2052,7 +2058,7 @@
       <c r="K20" s="25"/>
       <c r="L20" s="25"/>
     </row>
-    <row r="21" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="49.5">
       <c r="A21" t="s">
         <v>85</v>
       </c>
@@ -2084,7 +2090,7 @@
       </c>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="66">
       <c r="A22" t="s">
         <v>85</v>
       </c>
@@ -2114,7 +2120,7 @@
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="33">
       <c r="A23" t="s">
         <v>85</v>
       </c>
@@ -2142,7 +2148,7 @@
       <c r="K23" s="5"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="16.5">
       <c r="A24" t="s">
         <v>85</v>
       </c>
@@ -2166,7 +2172,7 @@
       </c>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="66">
       <c r="A25" t="s">
         <v>85</v>
       </c>
@@ -2192,7 +2198,7 @@
       </c>
       <c r="L25" s="8"/>
     </row>
-    <row r="26" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="66">
       <c r="A26" t="s">
         <v>85</v>
       </c>
@@ -2214,7 +2220,7 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
     </row>
-    <row r="27" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="66">
       <c r="A27" t="s">
         <v>85</v>
       </c>
@@ -2236,7 +2242,7 @@
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="49.5">
       <c r="A28" t="s">
         <v>85</v>
       </c>
@@ -2266,7 +2272,7 @@
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="66">
       <c r="A29" t="s">
         <v>85</v>
       </c>
@@ -2296,7 +2302,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="99">
       <c r="A30" t="s">
         <v>85</v>
       </c>
@@ -2326,7 +2332,7 @@
       </c>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="49.5">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -2356,7 +2362,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="49.5">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -2388,7 +2394,7 @@
       </c>
       <c r="L32" s="49"/>
     </row>
-    <row r="33" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="82.5">
       <c r="A33" t="s">
         <v>85</v>
       </c>
@@ -2419,7 +2425,7 @@
       </c>
       <c r="L33" s="52"/>
     </row>
-    <row r="34" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="49.5">
       <c r="A34" t="s">
         <v>85</v>
       </c>
@@ -2449,7 +2455,7 @@
       <c r="K34" s="51"/>
       <c r="L34" s="50"/>
     </row>
-    <row r="35" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" ht="82.5">
       <c r="A35" t="s">
         <v>85</v>
       </c>
@@ -2466,14 +2472,18 @@
       <c r="F35" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="G35" s="9"/>
-      <c r="H35" s="50"/>
+      <c r="G35" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>189</v>
+      </c>
       <c r="I35" s="8"/>
       <c r="J35" s="9"/>
       <c r="K35" s="13"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="115.5">
       <c r="A36" t="s">
         <v>85</v>
       </c>
@@ -2497,7 +2507,7 @@
       </c>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="66">
       <c r="B37" s="10"/>
       <c r="C37" s="5" t="s">
         <v>11</v>
@@ -2522,7 +2532,7 @@
       </c>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" ht="99">
       <c r="B38" s="10"/>
       <c r="C38" s="5" t="s">
         <v>18</v>
@@ -2541,7 +2551,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="115.5">
       <c r="B39" s="4">
         <v>11</v>
       </c>
@@ -2564,7 +2574,7 @@
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" ht="99">
       <c r="B40" s="10"/>
       <c r="C40" s="5" t="s">
         <v>11</v>
@@ -2591,7 +2601,7 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="49.5">
       <c r="B41" s="10"/>
       <c r="C41" s="9" t="s">
         <v>18</v>
@@ -2610,7 +2620,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="82.5">
       <c r="B42" s="4">
         <v>12</v>
       </c>
@@ -2635,7 +2645,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="82.5">
       <c r="B43" s="10"/>
       <c r="C43" s="5" t="s">
         <v>11</v>
@@ -2660,7 +2670,7 @@
       </c>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="82.5">
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
         <v>56</v>
@@ -2679,7 +2689,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="33">
       <c r="B45" s="4">
         <v>13</v>
       </c>
@@ -2704,7 +2714,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="99">
       <c r="B46" s="10"/>
       <c r="C46" s="5" t="s">
         <v>11</v>
@@ -2723,7 +2733,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" ht="66">
       <c r="B47" s="10"/>
       <c r="C47" s="9" t="s">
         <v>18</v>
@@ -2740,7 +2750,7 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" ht="148.5">
       <c r="B48" s="4">
         <v>14</v>
       </c>
@@ -2767,7 +2777,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="49" spans="2:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:12" ht="33">
       <c r="B49" s="10"/>
       <c r="C49" s="5" t="s">
         <v>11</v>
@@ -2792,7 +2802,7 @@
       </c>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="2:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:12" ht="49.5">
       <c r="B50" s="10"/>
       <c r="C50" s="9" t="s">
         <v>18</v>
@@ -2809,7 +2819,7 @@
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:12" ht="82.5">
       <c r="B51" s="10"/>
       <c r="C51" s="5" t="s">
         <v>72</v>
@@ -2830,7 +2840,7 @@
       <c r="K51" s="13"/>
       <c r="L51" s="8"/>
     </row>
-    <row r="52" spans="2:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:12" ht="16.5">
       <c r="B52" s="4">
         <v>15</v>
       </c>
@@ -2851,7 +2861,7 @@
       <c r="K52" s="8"/>
       <c r="L52" s="8"/>
     </row>
-    <row r="53" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:12" ht="99">
       <c r="B53" s="10"/>
       <c r="C53" s="5" t="s">
         <v>11</v>
@@ -2872,7 +2882,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="54" spans="2:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:12" ht="66">
       <c r="B54" s="10"/>
       <c r="C54" s="9" t="s">
         <v>18</v>
@@ -2891,7 +2901,7 @@
       <c r="K54" s="13"/>
       <c r="L54" s="8"/>
     </row>
-    <row r="55" spans="2:12" ht="165" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:12" ht="115.5">
       <c r="B55" s="4" t="s">
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
Added second logistic inference
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D411CE99-8607-4226-ADEE-2C354F2203BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8EA424-9DAF-4B92-A873-292B14EEE628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="195">
   <si>
     <t>week</t>
   </si>
@@ -144,18 +144,9 @@
     <t>Logistic regression: Comparing models</t>
   </si>
   <si>
-    <t>/slides/19-logistic-compare.html</t>
-  </si>
-  <si>
-    <t>/ae/ae-14-logistic-compare.html</t>
-  </si>
-  <si>
     <t>/hw/hw-04.html</t>
   </si>
   <si>
-    <t>HW 04 assigned</t>
-  </si>
-  <si>
     <t>Lab: Work on project</t>
   </si>
   <si>
@@ -600,9 +591,6 @@
     <t>/slides/26-logistic-estimation.html</t>
   </si>
   <si>
-    <t>HW 09 Due/ HW 10 Assigned</t>
-  </si>
-  <si>
     <t>Logistic regression: Conditions</t>
   </si>
   <si>
@@ -613,13 +601,31 @@
   </si>
   <si>
     <t>/slides/28-logistic-inference.html</t>
+  </si>
+  <si>
+    <t>/slides/29-logistic-inference2.html</t>
+  </si>
+  <si>
+    <t>/ae/ae-22-logistic-inference2.html</t>
+  </si>
+  <si>
+    <t>HW 09 Due</t>
+  </si>
+  <si>
+    <t>Logistic regression: Multiple Covariates</t>
+  </si>
+  <si>
+    <t>Rough Draft of Paper Due</t>
+  </si>
+  <si>
+    <t>/project-instructions.html#draft-report</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,14 +689,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -1117,9 +1115,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
@@ -1129,10 +1124,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1151,6 +1146,9 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -1501,7 +1499,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="16.5">
       <c r="A1" s="17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1539,7 +1537,7 @@
     </row>
     <row r="2" spans="1:12" ht="49.5">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
@@ -1558,17 +1556,17 @@
         <v>13</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
       <c r="L2" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="33">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="5" t="s">
@@ -1581,7 +1579,7 @@
         <v>16</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
@@ -1590,12 +1588,12 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="L3" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="66">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B4" s="4">
         <v>2</v>
@@ -1607,10 +1605,10 @@
         <v>45530</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
@@ -1619,7 +1617,7 @@
     </row>
     <row r="5" spans="1:12" ht="66">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="5" t="s">
@@ -1635,7 +1633,7 @@
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
@@ -1645,7 +1643,7 @@
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>22</v>
@@ -1653,7 +1651,7 @@
     </row>
     <row r="6" spans="1:12" ht="49.5">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="5" t="s">
@@ -1663,14 +1661,14 @@
         <v>45534</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -1679,7 +1677,7 @@
     </row>
     <row r="7" spans="1:12" ht="16.5">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B7" s="4">
         <v>3</v>
@@ -1691,12 +1689,12 @@
         <v>45537</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="99">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5" t="s">
@@ -1709,26 +1707,26 @@
         <v>23</v>
       </c>
       <c r="F8" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>94</v>
-      </c>
       <c r="H8" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>29</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L8" s="8"/>
     </row>
     <row r="9" spans="1:12" ht="165">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="5" t="s">
@@ -1738,21 +1736,21 @@
         <v>45541</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="8"/>
       <c r="K9" s="9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>26</v>
@@ -1760,7 +1758,7 @@
     </row>
     <row r="10" spans="1:12" ht="115.5">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B10" s="4">
         <v>4</v>
@@ -1775,10 +1773,10 @@
         <v>27</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="8"/>
@@ -1788,7 +1786,7 @@
     </row>
     <row r="11" spans="1:12" ht="148.5">
       <c r="A11" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="5" t="s">
@@ -1798,14 +1796,14 @@
         <v>45546</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="5"/>
@@ -1813,7 +1811,7 @@
     </row>
     <row r="12" spans="1:12" ht="66">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="5" t="s">
@@ -1826,26 +1824,26 @@
         <v>28</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I12" s="31" t="s">
         <v>32</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L12" s="8"/>
     </row>
     <row r="13" spans="1:12" ht="99">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B13" s="32">
         <v>5</v>
@@ -1857,16 +1855,16 @@
         <v>45551</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I13" s="37"/>
       <c r="J13" s="35"/>
@@ -1875,7 +1873,7 @@
     </row>
     <row r="14" spans="1:12" ht="66">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="33" t="s">
@@ -1885,16 +1883,16 @@
         <v>45553</v>
       </c>
       <c r="E14" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="35"/>
@@ -1903,7 +1901,7 @@
     </row>
     <row r="15" spans="1:12" ht="49.5">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B15" s="32"/>
       <c r="C15" s="33" t="s">
@@ -1913,29 +1911,29 @@
         <v>45555</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I15" s="37" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J15" s="35"/>
       <c r="K15" s="36" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L15" s="35"/>
     </row>
     <row r="16" spans="1:12" ht="49.5">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" s="32">
         <v>6</v>
@@ -1947,25 +1945,25 @@
         <v>45558</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G16" s="36"/>
       <c r="H16" s="39"/>
       <c r="I16" s="37"/>
-      <c r="J16" s="41" t="s">
+      <c r="J16" s="52" t="s">
         <v>33</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="L16" s="35"/>
     </row>
     <row r="17" spans="1:12" ht="99">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="33" t="s">
@@ -1975,7 +1973,7 @@
         <v>45560</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="35"/>
@@ -1984,7 +1982,7 @@
     </row>
     <row r="18" spans="1:12" ht="33">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="33" t="s">
@@ -1994,29 +1992,29 @@
         <v>45562</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G18" s="36" t="s">
+        <v>116</v>
+      </c>
+      <c r="H18" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="H18" s="39" t="s">
-        <v>122</v>
-      </c>
       <c r="I18" s="37" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J18" s="35"/>
       <c r="K18" s="24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L18" s="35"/>
     </row>
     <row r="19" spans="1:12" ht="66">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B19" s="4">
         <v>7</v>
@@ -2028,16 +2026,16 @@
         <v>45565</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="F19" s="45" t="s">
-        <v>131</v>
+        <v>110</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>128</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I19" s="24"/>
       <c r="J19" s="24"/>
@@ -2045,26 +2043,26 @@
     </row>
     <row r="20" spans="1:12" ht="66">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B20" s="20"/>
-      <c r="C20" s="43" t="s">
+      <c r="C20" s="42" t="s">
         <v>11</v>
       </c>
       <c r="D20" s="23">
         <v>45567</v>
       </c>
       <c r="E20" s="40" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" s="45" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>131</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
@@ -2073,60 +2071,60 @@
     </row>
     <row r="21" spans="1:12" ht="49.5">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B21" s="10"/>
-      <c r="C21" s="42" t="s">
+      <c r="C21" s="41" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="23">
         <v>45569</v>
       </c>
-      <c r="E21" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="F21" s="46" t="s">
-        <v>144</v>
+      <c r="E21" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="F21" s="45" t="s">
+        <v>141</v>
       </c>
       <c r="G21" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="I21" s="9" t="s">
         <v>135</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>138</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="L21" s="8"/>
     </row>
     <row r="22" spans="1:12" ht="66">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B22" s="4">
         <v>8</v>
       </c>
-      <c r="C22" s="47" t="s">
+      <c r="C22" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="48">
+      <c r="D22" s="47">
         <v>45572</v>
       </c>
-      <c r="E22" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="F22" s="46" t="s">
+      <c r="E22" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="F22" s="45" t="s">
+        <v>140</v>
+      </c>
+      <c r="G22" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="H22" s="27" t="s">
         <v>143</v>
-      </c>
-      <c r="G22" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>146</v>
       </c>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
@@ -2135,7 +2133,7 @@
     </row>
     <row r="23" spans="1:12" ht="33">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="5" t="s">
@@ -2148,13 +2146,13 @@
         <v>30</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
@@ -2163,7 +2161,7 @@
     </row>
     <row r="24" spans="1:12" ht="16.5">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="5" t="s">
@@ -2181,13 +2179,13 @@
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="L24" s="8"/>
     </row>
     <row r="25" spans="1:12" ht="66">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B25" s="4">
         <v>9</v>
@@ -2199,7 +2197,7 @@
         <v>45579</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -2207,13 +2205,13 @@
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="L25" s="8"/>
     </row>
     <row r="26" spans="1:12" ht="66">
       <c r="A26" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="9" t="s">
@@ -2223,7 +2221,7 @@
         <v>45581</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -2235,7 +2233,7 @@
     </row>
     <row r="27" spans="1:12" ht="66">
       <c r="A27" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="5" t="s">
@@ -2245,7 +2243,7 @@
         <v>45583</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
@@ -2257,7 +2255,7 @@
     </row>
     <row r="28" spans="1:12" ht="49.5">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B28" s="4">
         <v>10</v>
@@ -2269,16 +2267,16 @@
         <v>45586</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I28" s="13"/>
       <c r="J28" s="8"/>
@@ -2287,7 +2285,7 @@
     </row>
     <row r="29" spans="1:12" ht="66">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="9" t="s">
@@ -2297,27 +2295,27 @@
         <v>45588</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="G29" s="26" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
       <c r="L29" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="99">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="5" t="s">
@@ -2327,27 +2325,27 @@
         <v>45590</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="26" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="L30" s="8"/>
     </row>
     <row r="31" spans="1:12" ht="49.5">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B31" s="4">
         <v>11</v>
@@ -2359,16 +2357,16 @@
         <v>45593</v>
       </c>
       <c r="E31" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="G31" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>165</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
@@ -2377,7 +2375,7 @@
     </row>
     <row r="32" spans="1:12" ht="49.5">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="9" t="s">
@@ -2387,29 +2385,29 @@
         <v>45595</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F32" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G32" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="G32" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="I32" s="49"/>
-      <c r="J32" s="52" t="s">
-        <v>161</v>
-      </c>
-      <c r="K32" s="49" t="s">
-        <v>162</v>
-      </c>
-      <c r="L32" s="49"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="K32" s="48" t="s">
+        <v>159</v>
+      </c>
+      <c r="L32" s="48"/>
     </row>
     <row r="33" spans="1:12" ht="82.5">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="5" t="s">
@@ -2419,28 +2417,28 @@
         <v>45597</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F33" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G33" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="G33" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>172</v>
-      </c>
       <c r="I33" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="K33" s="52" t="s">
-        <v>160</v>
-      </c>
-      <c r="L33" s="52"/>
+        <v>174</v>
+      </c>
+      <c r="K33" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="L33" s="51"/>
     </row>
     <row r="34" spans="1:12" ht="49.5">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B34" s="4">
         <v>12</v>
@@ -2455,22 +2453,22 @@
         <v>34</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G34" s="26" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="I34" s="51"/>
-      <c r="J34" s="50"/>
-      <c r="K34" s="51"/>
-      <c r="L34" s="50"/>
+        <v>172</v>
+      </c>
+      <c r="I34" s="50"/>
+      <c r="J34" s="49"/>
+      <c r="K34" s="50"/>
+      <c r="L34" s="49"/>
     </row>
     <row r="35" spans="1:12" ht="82.5">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="9" t="s">
@@ -2480,16 +2478,16 @@
         <v>45602</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G35" s="26" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I35" s="8"/>
       <c r="J35" s="9"/>
@@ -2498,7 +2496,7 @@
     </row>
     <row r="36" spans="1:12" ht="82.5">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="5" t="s">
@@ -2508,26 +2506,26 @@
         <v>45604</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G36" s="26" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="J36" s="8"/>
-      <c r="K36" s="52" t="s">
-        <v>179</v>
+      <c r="K36" s="51" t="s">
+        <v>176</v>
       </c>
       <c r="L36" s="8"/>
     </row>
     <row r="37" spans="1:12" ht="82.5">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B37" s="4">
         <v>13</v>
@@ -2539,13 +2537,13 @@
         <v>45607</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G37" s="26" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="H37" s="9"/>
       <c r="I37" s="8"/>
@@ -2555,7 +2553,7 @@
     </row>
     <row r="38" spans="1:12" ht="82.5">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="5" t="s">
@@ -2565,16 +2563,16 @@
         <v>45609</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G38" s="26" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I38" s="8"/>
       <c r="J38" s="8"/>
@@ -2583,7 +2581,7 @@
     </row>
     <row r="39" spans="1:12" ht="99">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="5" t="s">
@@ -2596,41 +2594,44 @@
         <v>35</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="G39" s="9"/>
-      <c r="H39" s="13"/>
+        <v>182</v>
+      </c>
+      <c r="G39" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>190</v>
+      </c>
       <c r="I39" s="8"/>
       <c r="J39" s="8"/>
       <c r="K39" s="8" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="L39" s="8"/>
     </row>
     <row r="40" spans="1:12" ht="99">
+      <c r="A40" t="s">
+        <v>75</v>
+      </c>
       <c r="B40" s="10"/>
       <c r="C40" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D40" s="6">
-        <v>45604</v>
+        <v>45613</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>35</v>
+        <v>192</v>
       </c>
       <c r="F40" s="8"/>
-      <c r="G40" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I40" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="J40" s="8"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="8" t="s">
+        <v>194</v>
+      </c>
       <c r="K40" s="9" t="s">
-        <v>39</v>
+        <v>193</v>
       </c>
       <c r="L40" s="8"/>
     </row>
@@ -2641,7 +2642,7 @@
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
@@ -2650,7 +2651,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="82.5">
@@ -2664,14 +2665,14 @@
         <v>45609</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F42" s="8"/>
       <c r="G42" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>
@@ -2687,30 +2688,30 @@
         <v>45611</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="I43" s="13"/>
       <c r="J43" s="8"/>
       <c r="K43" s="15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="L43" s="8"/>
     </row>
     <row r="44" spans="1:12" ht="82.5">
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -2719,7 +2720,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="13"/>
       <c r="L44" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="33">
@@ -2733,17 +2734,17 @@
         <v>45616</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J45" s="8"/>
       <c r="K45" s="9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="L45" s="8"/>
     </row>
@@ -2756,7 +2757,7 @@
         <v>45618</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -2773,7 +2774,7 @@
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -2794,20 +2795,20 @@
         <v>45623</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H48" s="13"/>
       <c r="I48" s="8"/>
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
       <c r="L48" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="33">
@@ -2819,19 +2820,19 @@
         <v>45625</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I49" s="13"/>
       <c r="J49" s="8"/>
       <c r="K49" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="L49" s="8"/>
     </row>
@@ -2842,7 +2843,7 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
@@ -2855,20 +2856,20 @@
     <row r="51" spans="2:12" ht="82.5">
       <c r="B51" s="10"/>
       <c r="C51" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D51" s="6">
         <v>45627</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="8"/>
       <c r="J51" s="9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="K51" s="13"/>
       <c r="L51" s="8"/>
@@ -2884,7 +2885,7 @@
         <v>45630</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
@@ -2903,7 +2904,7 @@
         <v>45632</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
@@ -2912,7 +2913,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
       <c r="L53" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="2:12" ht="66">
@@ -2922,39 +2923,39 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
       <c r="J54" s="16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="K54" s="13"/>
       <c r="L54" s="8"/>
     </row>
     <row r="55" spans="2:12" ht="115.5">
       <c r="B55" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C55" s="8"/>
       <c r="D55" s="6">
         <v>45639</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
       <c r="J55" s="16" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K55" s="8"/>
       <c r="L55" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added mutiple logistic regression reading
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283C30C4-2C62-4A19-B0FA-9CBE2D4A467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4AE7BE-2DF7-4BF9-8581-91EEC6BC43B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="196">
   <si>
     <t>week</t>
   </si>
@@ -609,9 +609,6 @@
     <t>HW 09 Due</t>
   </si>
   <si>
-    <t>Logistic regression: Multiple Covariates</t>
-  </si>
-  <si>
     <t>Rough Draft of Paper Due</t>
   </si>
   <si>
@@ -619,6 +616,12 @@
   </si>
   <si>
     <t>Logistic regression: Inference Continued</t>
+  </si>
+  <si>
+    <t>/prepare/multiple-logistic-regression.html</t>
+  </si>
+  <si>
+    <t>Multiple Logistic Regression</t>
   </si>
 </sst>
 </file>
@@ -2591,7 +2594,7 @@
         <v>45611</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>181</v>
@@ -2609,7 +2612,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="99">
+    <row r="40" spans="1:12" ht="66">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -2620,29 +2623,33 @@
         <v>19</v>
       </c>
       <c r="D40" s="6">
-        <v>45613</v>
+        <v>45614</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="F40" s="8"/>
+        <v>195</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
       <c r="I40" s="9"/>
       <c r="J40" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L40" s="8"/>
     </row>
     <row r="41" spans="1:12" ht="49.5">
       <c r="B41" s="10"/>
       <c r="C41" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="8"/>
+        <v>11</v>
+      </c>
+      <c r="D41" s="6">
+        <v>45616</v>
+      </c>
       <c r="E41" s="7" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Added Multiple logistic regression
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C402190D-61C1-46CF-AC3D-1989B2303D0E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="200">
   <si>
     <t>week</t>
   </si>
@@ -606,9 +606,6 @@
     <t>HW 09 Due</t>
   </si>
   <si>
-    <t>Rough Draft of Paper Due</t>
-  </si>
-  <si>
     <t>/project-instructions.html#draft-report</t>
   </si>
   <si>
@@ -622,13 +619,28 @@
   </si>
   <si>
     <t>/slides/27-logistic-conditions.html</t>
+  </si>
+  <si>
+    <t>/slides/30-logistic-multiple.html</t>
+  </si>
+  <si>
+    <t>/ae/ae-23-multiple-logistic.html</t>
+  </si>
+  <si>
+    <t>/prepare/logistic-model-selection.html</t>
+  </si>
+  <si>
+    <t>Rough Draft of Paper Due/ HW 10 Assigned</t>
+  </si>
+  <si>
+    <t>LR: Model Selection and Transformations</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1151,7 +1163,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -1495,12 +1507,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C666FC1-734D-4F31-9D28-5509B94BC597}">
   <dimension ref="A1:L55"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>73</v>
       </c>
@@ -1538,7 +1550,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="49.5">
+    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -1567,7 +1579,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="33">
+    <row r="3" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>74</v>
       </c>
@@ -1594,7 +1606,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="66">
+    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -1618,7 +1630,7 @@
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
     </row>
-    <row r="5" spans="1:12" ht="66">
+    <row r="5" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>74</v>
       </c>
@@ -1652,7 +1664,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="49.5">
+    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -1678,7 +1690,7 @@
       <c r="K6" s="28"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="16.5">
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>74</v>
       </c>
@@ -1695,7 +1707,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="99">
+    <row r="8" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>74</v>
       </c>
@@ -1727,7 +1739,7 @@
       </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="165">
+    <row r="9" spans="1:12" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>74</v>
       </c>
@@ -1759,7 +1771,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="115.5">
+    <row r="10" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>74</v>
       </c>
@@ -1787,7 +1799,7 @@
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" ht="148.5">
+    <row r="11" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>74</v>
       </c>
@@ -1812,7 +1824,7 @@
       <c r="K11" s="5"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" ht="66">
+    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>74</v>
       </c>
@@ -1844,7 +1856,7 @@
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" ht="99">
+    <row r="13" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1874,7 +1886,7 @@
       <c r="K13" s="36"/>
       <c r="L13" s="35"/>
     </row>
-    <row r="14" spans="1:12" ht="66">
+    <row r="14" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>74</v>
       </c>
@@ -1902,7 +1914,7 @@
       <c r="K14" s="36"/>
       <c r="L14" s="35"/>
     </row>
-    <row r="15" spans="1:12" ht="49.5">
+    <row r="15" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -1934,7 +1946,7 @@
       </c>
       <c r="L15" s="35"/>
     </row>
-    <row r="16" spans="1:12" ht="49.5">
+    <row r="16" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -1964,7 +1976,7 @@
       </c>
       <c r="L16" s="35"/>
     </row>
-    <row r="17" spans="1:12" ht="99">
+    <row r="17" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>74</v>
       </c>
@@ -1983,7 +1995,7 @@
       <c r="K17" s="36"/>
       <c r="L17" s="35"/>
     </row>
-    <row r="18" spans="1:12" ht="33">
+    <row r="18" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>74</v>
       </c>
@@ -2015,7 +2027,7 @@
       </c>
       <c r="L18" s="35"/>
     </row>
-    <row r="19" spans="1:12" ht="66">
+    <row r="19" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>74</v>
       </c>
@@ -2044,7 +2056,7 @@
       <c r="J19" s="24"/>
       <c r="L19" s="24"/>
     </row>
-    <row r="20" spans="1:12" ht="66">
+    <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -2072,7 +2084,7 @@
       <c r="K20" s="25"/>
       <c r="L20" s="25"/>
     </row>
-    <row r="21" spans="1:12" ht="49.5">
+    <row r="21" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -2104,7 +2116,7 @@
       </c>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" ht="66">
+    <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -2134,7 +2146,7 @@
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" ht="33">
+    <row r="23" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -2162,7 +2174,7 @@
       <c r="K23" s="5"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" ht="16.5">
+    <row r="24" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -2186,7 +2198,7 @@
       </c>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" ht="66">
+    <row r="25" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>74</v>
       </c>
@@ -2212,7 +2224,7 @@
       </c>
       <c r="L25" s="8"/>
     </row>
-    <row r="26" spans="1:12" ht="66">
+    <row r="26" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -2234,7 +2246,7 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
     </row>
-    <row r="27" spans="1:12" ht="66">
+    <row r="27" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>74</v>
       </c>
@@ -2256,7 +2268,7 @@
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" ht="49.5">
+    <row r="28" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>74</v>
       </c>
@@ -2286,7 +2298,7 @@
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" ht="66">
+    <row r="29" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>74</v>
       </c>
@@ -2316,7 +2328,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="99">
+    <row r="30" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>74</v>
       </c>
@@ -2346,7 +2358,7 @@
       </c>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" ht="49.5">
+    <row r="31" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -2376,7 +2388,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" ht="49.5">
+    <row r="32" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -2408,7 +2420,7 @@
       </c>
       <c r="L32" s="48"/>
     </row>
-    <row r="33" spans="1:12" ht="82.5">
+    <row r="33" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -2439,7 +2451,7 @@
       </c>
       <c r="L33" s="51"/>
     </row>
-    <row r="34" spans="1:12" ht="49.5">
+    <row r="34" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -2469,7 +2481,7 @@
       <c r="K34" s="50"/>
       <c r="L34" s="49"/>
     </row>
-    <row r="35" spans="1:12" ht="82.5">
+    <row r="35" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -2497,7 +2509,7 @@
       <c r="K35" s="13"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" ht="82.5">
+    <row r="36" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>74</v>
       </c>
@@ -2526,7 +2538,7 @@
       </c>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" ht="82.5">
+    <row r="37" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2546,7 +2558,7 @@
         <v>178</v>
       </c>
       <c r="G37" s="26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H37" s="9"/>
       <c r="I37" s="8"/>
@@ -2554,7 +2566,7 @@
       <c r="K37" s="5"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" ht="82.5">
+    <row r="38" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -2582,7 +2594,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" ht="115.5">
+    <row r="39" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -2594,7 +2606,7 @@
         <v>45611</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>181</v>
@@ -2612,7 +2624,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="66">
+    <row r="40" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -2626,23 +2638,30 @@
         <v>45614</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
+        <v>192</v>
+      </c>
+      <c r="G40" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>196</v>
+      </c>
       <c r="I40" s="9"/>
       <c r="J40" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="49.5">
+    <row r="41" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>74</v>
+      </c>
       <c r="B41" s="10"/>
       <c r="C41" s="9" t="s">
         <v>11</v>
@@ -2651,9 +2670,11 @@
         <v>45616</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F41" s="8"/>
+        <v>199</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>197</v>
+      </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
       <c r="I41" s="8"/>
@@ -2663,7 +2684,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="82.5">
+    <row r="42" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B42" s="4">
         <v>12</v>
       </c>
@@ -2688,7 +2709,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="82.5">
+    <row r="43" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B43" s="10"/>
       <c r="C43" s="5" t="s">
         <v>11</v>
@@ -2713,7 +2734,7 @@
       </c>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="82.5">
+    <row r="44" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
         <v>45</v>
@@ -2732,7 +2753,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="33">
+    <row r="45" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B45" s="4">
         <v>13</v>
       </c>
@@ -2757,7 +2778,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="99">
+    <row r="46" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="B46" s="10"/>
       <c r="C46" s="5" t="s">
         <v>11</v>
@@ -2776,7 +2797,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" ht="66">
+    <row r="47" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B47" s="10"/>
       <c r="C47" s="9" t="s">
         <v>18</v>
@@ -2793,7 +2814,7 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" spans="1:12" ht="148.5">
+    <row r="48" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
       <c r="B48" s="4">
         <v>14</v>
       </c>
@@ -2820,7 +2841,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="2:12" ht="33">
+    <row r="49" spans="2:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B49" s="10"/>
       <c r="C49" s="5" t="s">
         <v>11</v>
@@ -2845,7 +2866,7 @@
       </c>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="2:12" ht="49.5">
+    <row r="50" spans="2:12" ht="66" x14ac:dyDescent="0.3">
       <c r="B50" s="10"/>
       <c r="C50" s="9" t="s">
         <v>18</v>
@@ -2862,7 +2883,7 @@
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="2:12" ht="82.5">
+    <row r="51" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="B51" s="10"/>
       <c r="C51" s="5" t="s">
         <v>61</v>
@@ -2883,7 +2904,7 @@
       <c r="K51" s="13"/>
       <c r="L51" s="8"/>
     </row>
-    <row r="52" spans="2:12" ht="16.5">
+    <row r="52" spans="2:12" ht="33" x14ac:dyDescent="0.3">
       <c r="B52" s="4">
         <v>15</v>
       </c>
@@ -2904,7 +2925,7 @@
       <c r="K52" s="8"/>
       <c r="L52" s="8"/>
     </row>
-    <row r="53" spans="2:12" ht="99">
+    <row r="53" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="B53" s="10"/>
       <c r="C53" s="5" t="s">
         <v>11</v>
@@ -2925,7 +2946,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="2:12" ht="66">
+    <row r="54" spans="2:12" ht="66" x14ac:dyDescent="0.3">
       <c r="B54" s="10"/>
       <c r="C54" s="9" t="s">
         <v>18</v>
@@ -2944,7 +2965,7 @@
       <c r="K54" s="13"/>
       <c r="L54" s="8"/>
     </row>
-    <row r="55" spans="2:12" ht="115.5">
+    <row r="55" spans="2:12" ht="165" x14ac:dyDescent="0.3">
       <c r="B55" s="4" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
Added hw 10 and extra days to calendar
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C402190D-61C1-46CF-AC3D-1989B2303D0E}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CFB1A67-2111-470D-88E9-BC0B17A3CC04}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="194">
   <si>
     <t>week</t>
   </si>
@@ -147,48 +147,12 @@
     <t>Lab: Work on project</t>
   </si>
   <si>
-    <t>Last day to withdraw with W 11/5</t>
-  </si>
-  <si>
     <t>Logistic regression: Inference</t>
   </si>
   <si>
-    <t>/slides/20-logistic-inf.html</t>
-  </si>
-  <si>
-    <t>/ae/ae-15-logistic-inference.html</t>
-  </si>
-  <si>
-    <t>Mulitnomial logistic regression</t>
-  </si>
-  <si>
-    <t>/slides/21-multinomial-logistic.html</t>
-  </si>
-  <si>
-    <t>/ae/ae-16-logistic-conditions.html</t>
-  </si>
-  <si>
-    <t>HW 04 due</t>
-  </si>
-  <si>
-    <t>Tu &amp;Th</t>
-  </si>
-  <si>
-    <t>Lab: Project draft peer review</t>
-  </si>
-  <si>
-    <t>(do partially in class?)</t>
-  </si>
-  <si>
-    <t>Project work day</t>
-  </si>
-  <si>
     <t>/hw/hw-05.html</t>
   </si>
   <si>
-    <t>Statistics experience due, HW 05 assigned</t>
-  </si>
-  <si>
     <t>NO LECTURE: Thanksgiving Break</t>
   </si>
   <si>
@@ -634,6 +598,24 @@
   </si>
   <si>
     <t>LR: Model Selection and Transformations</t>
+  </si>
+  <si>
+    <t>/hw/hw-10.html</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>Peer Review Due/HW 10 Due</t>
+  </si>
+  <si>
+    <t>Exam Review</t>
+  </si>
+  <si>
+    <t>Exam 2</t>
+  </si>
+  <si>
+    <t>/project-instructions.html#peer-review</t>
   </si>
 </sst>
 </file>
@@ -1506,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C666FC1-734D-4F31-9D28-5509B94BC597}">
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
@@ -1514,7 +1496,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1552,7 +1534,7 @@
     </row>
     <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
@@ -1571,17 +1553,17 @@
         <v>13</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
       <c r="L2" s="5" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="5" t="s">
@@ -1594,7 +1576,7 @@
         <v>16</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
@@ -1603,12 +1585,12 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="L3" s="5" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B4" s="4">
         <v>2</v>
@@ -1620,10 +1602,10 @@
         <v>45530</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
@@ -1632,7 +1614,7 @@
     </row>
     <row r="5" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="5" t="s">
@@ -1648,7 +1630,7 @@
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
@@ -1658,7 +1640,7 @@
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>22</v>
@@ -1666,7 +1648,7 @@
     </row>
     <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="5" t="s">
@@ -1676,14 +1658,14 @@
         <v>45534</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -1692,7 +1674,7 @@
     </row>
     <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B7" s="4">
         <v>3</v>
@@ -1704,12 +1686,12 @@
         <v>45537</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5" t="s">
@@ -1722,26 +1704,26 @@
         <v>23</v>
       </c>
       <c r="F8" s="30" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>29</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="L8" s="8"/>
     </row>
     <row r="9" spans="1:12" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="5" t="s">
@@ -1751,21 +1733,21 @@
         <v>45541</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="8"/>
       <c r="K9" s="9" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>26</v>
@@ -1773,7 +1755,7 @@
     </row>
     <row r="10" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4">
         <v>4</v>
@@ -1788,10 +1770,10 @@
         <v>27</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="8"/>
@@ -1801,7 +1783,7 @@
     </row>
     <row r="11" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="5" t="s">
@@ -1811,14 +1793,14 @@
         <v>45546</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="5" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="5"/>
@@ -1826,7 +1808,7 @@
     </row>
     <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="5" t="s">
@@ -1839,26 +1821,26 @@
         <v>28</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="I12" s="31" t="s">
         <v>32</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="L12" s="8"/>
     </row>
     <row r="13" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B13" s="32">
         <v>5</v>
@@ -1870,16 +1852,16 @@
         <v>45551</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="I13" s="37"/>
       <c r="J13" s="35"/>
@@ -1888,7 +1870,7 @@
     </row>
     <row r="14" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B14" s="32"/>
       <c r="C14" s="33" t="s">
@@ -1898,16 +1880,16 @@
         <v>45553</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="I14" s="37"/>
       <c r="J14" s="35"/>
@@ -1916,7 +1898,7 @@
     </row>
     <row r="15" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B15" s="32"/>
       <c r="C15" s="33" t="s">
@@ -1926,29 +1908,29 @@
         <v>45555</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="I15" s="37" t="s">
         <v>35</v>
       </c>
       <c r="J15" s="35"/>
       <c r="K15" s="36" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="L15" s="35"/>
     </row>
     <row r="16" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B16" s="32">
         <v>6</v>
@@ -1960,10 +1942,10 @@
         <v>45558</v>
       </c>
       <c r="E16" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="35" t="s">
         <v>108</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>120</v>
       </c>
       <c r="G16" s="36"/>
       <c r="H16" s="39"/>
@@ -1972,13 +1954,13 @@
         <v>33</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="L16" s="35"/>
     </row>
     <row r="17" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="33" t="s">
@@ -1988,7 +1970,7 @@
         <v>45560</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I17" s="37"/>
       <c r="J17" s="35"/>
@@ -1997,7 +1979,7 @@
     </row>
     <row r="18" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="33" t="s">
@@ -2007,29 +1989,29 @@
         <v>45562</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="H18" s="39" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="J18" s="35"/>
       <c r="K18" s="24" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="L18" s="35"/>
     </row>
     <row r="19" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B19" s="4">
         <v>7</v>
@@ -2041,16 +2023,16 @@
         <v>45565</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="F19" s="44" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I19" s="24"/>
       <c r="J19" s="24"/>
@@ -2058,7 +2040,7 @@
     </row>
     <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="42" t="s">
@@ -2068,16 +2050,16 @@
         <v>45567</v>
       </c>
       <c r="E20" s="40" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="F20" s="44" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
@@ -2086,7 +2068,7 @@
     </row>
     <row r="21" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="41" t="s">
@@ -2096,29 +2078,29 @@
         <v>45569</v>
       </c>
       <c r="E21" s="43" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="F21" s="45" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="H21" s="27" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="8" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="L21" s="8"/>
     </row>
     <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B22" s="4">
         <v>8</v>
@@ -2130,16 +2112,16 @@
         <v>45572</v>
       </c>
       <c r="E22" s="43" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="F22" s="45" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
@@ -2148,7 +2130,7 @@
     </row>
     <row r="23" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="5" t="s">
@@ -2161,13 +2143,13 @@
         <v>30</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
@@ -2176,7 +2158,7 @@
     </row>
     <row r="24" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="5" t="s">
@@ -2194,13 +2176,13 @@
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="L24" s="8"/>
     </row>
     <row r="25" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B25" s="4">
         <v>9</v>
@@ -2212,7 +2194,7 @@
         <v>45579</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -2220,13 +2202,13 @@
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="L25" s="8"/>
     </row>
     <row r="26" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="9" t="s">
@@ -2236,7 +2218,7 @@
         <v>45581</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -2248,7 +2230,7 @@
     </row>
     <row r="27" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="5" t="s">
@@ -2258,7 +2240,7 @@
         <v>45583</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
@@ -2270,7 +2252,7 @@
     </row>
     <row r="28" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4">
         <v>10</v>
@@ -2282,16 +2264,16 @@
         <v>45586</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="I28" s="13"/>
       <c r="J28" s="8"/>
@@ -2300,7 +2282,7 @@
     </row>
     <row r="29" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="9" t="s">
@@ -2310,27 +2292,27 @@
         <v>45588</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="G29" s="26" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
       <c r="L29" s="5" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="5" t="s">
@@ -2340,27 +2322,27 @@
         <v>45590</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="26" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="L30" s="8"/>
     </row>
     <row r="31" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B31" s="4">
         <v>11</v>
@@ -2372,16 +2354,16 @@
         <v>45593</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="G31" s="26" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
@@ -2390,7 +2372,7 @@
     </row>
     <row r="32" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="9" t="s">
@@ -2400,29 +2382,29 @@
         <v>45595</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G32" s="26" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="I32" s="48"/>
       <c r="J32" s="51" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="K32" s="48" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="L32" s="48"/>
     </row>
     <row r="33" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="5" t="s">
@@ -2432,28 +2414,28 @@
         <v>45597</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G33" s="26" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="K33" s="51" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="L33" s="51"/>
     </row>
     <row r="34" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B34" s="4">
         <v>12</v>
@@ -2468,13 +2450,13 @@
         <v>34</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G34" s="26" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="I34" s="50"/>
       <c r="J34" s="49"/>
@@ -2483,7 +2465,7 @@
     </row>
     <row r="35" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="9" t="s">
@@ -2493,16 +2475,16 @@
         <v>45602</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G35" s="26" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="I35" s="8"/>
       <c r="J35" s="9"/>
@@ -2511,7 +2493,7 @@
     </row>
     <row r="36" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="5" t="s">
@@ -2521,26 +2503,26 @@
         <v>45604</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="G36" s="26" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="J36" s="8"/>
       <c r="K36" s="51" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="L36" s="8"/>
     </row>
     <row r="37" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B37" s="4">
         <v>13</v>
@@ -2552,13 +2534,13 @@
         <v>45607</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="G37" s="26" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="H37" s="9"/>
       <c r="I37" s="8"/>
@@ -2568,7 +2550,7 @@
     </row>
     <row r="38" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="5" t="s">
@@ -2578,16 +2560,16 @@
         <v>45609</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="G38" s="26" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="I38" s="8"/>
       <c r="J38" s="8"/>
@@ -2596,7 +2578,7 @@
     </row>
     <row r="39" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="5" t="s">
@@ -2606,27 +2588,27 @@
         <v>45611</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="G39" s="26" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="I39" s="8"/>
       <c r="J39" s="8"/>
       <c r="K39" s="8" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="L39" s="8"/>
     </row>
     <row r="40" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B40" s="4">
         <v>14</v>
@@ -2638,29 +2620,31 @@
         <v>45614</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="G40" s="26" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="I40" s="9"/>
+        <v>184</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>188</v>
+      </c>
       <c r="J40" s="8" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="L40" s="8"/>
     </row>
     <row r="41" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B41" s="10"/>
       <c r="C41" s="9" t="s">
@@ -2670,78 +2654,81 @@
         <v>45616</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
       <c r="I41" s="8"/>
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
-      <c r="L41" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="B42" s="4">
-        <v>12</v>
-      </c>
+      <c r="L41" s="5"/>
+    </row>
+    <row r="42" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>62</v>
+      </c>
+      <c r="B42" s="4"/>
       <c r="C42" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D42" s="6">
-        <v>45609</v>
+        <v>45618</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>38</v>
+        <v>189</v>
       </c>
       <c r="F42" s="8"/>
-      <c r="G42" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>40</v>
-      </c>
+      <c r="G42" s="5"/>
+      <c r="H42" s="9"/>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="B43" s="10"/>
+    <row r="43" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="4">
+        <v>15</v>
+      </c>
       <c r="C43" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D43" s="6">
-        <v>45611</v>
+        <v>45621</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>41</v>
+        <v>191</v>
       </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>43</v>
-      </c>
+      <c r="G43" s="5"/>
+      <c r="H43" s="9"/>
       <c r="I43" s="13"/>
-      <c r="J43" s="8"/>
+      <c r="J43" s="8" t="s">
+        <v>193</v>
+      </c>
       <c r="K43" s="15" t="s">
-        <v>44</v>
+        <v>190</v>
       </c>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>62</v>
+      </c>
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D44" s="8"/>
+        <v>11</v>
+      </c>
+      <c r="D44" s="6">
+        <v>45623</v>
+      </c>
       <c r="E44" s="7" t="s">
-        <v>46</v>
+        <v>192</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -2749,45 +2736,38 @@
       <c r="I44" s="8"/>
       <c r="J44" s="8"/>
       <c r="K44" s="13"/>
-      <c r="L44" s="12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B45" s="4">
-        <v>13</v>
-      </c>
+      <c r="L44" s="12"/>
+    </row>
+    <row r="45" spans="1:12" ht="86.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="10"/>
       <c r="C45" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D45" s="6">
-        <v>45616</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>48</v>
+        <v>45625</v>
+      </c>
+      <c r="E45" s="11" t="s">
+        <v>39</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
-      <c r="I45" s="9" t="s">
-        <v>49</v>
-      </c>
+      <c r="I45" s="8"/>
       <c r="J45" s="8"/>
-      <c r="K45" s="9" t="s">
-        <v>50</v>
-      </c>
+      <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B46" s="10"/>
-      <c r="C46" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="6">
-        <v>45618</v>
-      </c>
+      <c r="C46" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="8"/>
       <c r="E46" s="11" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -2797,125 +2777,127 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="B47" s="10"/>
-      <c r="C47" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
+    <row r="47" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
+      <c r="B47" s="4">
+        <v>14</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="6">
+        <v>45623</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H47" s="13"/>
       <c r="I47" s="8"/>
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
-    </row>
-    <row r="48" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
-      <c r="B48" s="4">
-        <v>14</v>
-      </c>
+      <c r="L47" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="B48" s="10"/>
       <c r="C48" s="5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D48" s="6">
-        <v>45623</v>
+        <v>45625</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="H48" s="13"/>
-      <c r="I48" s="8"/>
+        <v>45</v>
+      </c>
+      <c r="F48" s="8"/>
+      <c r="G48" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H48" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I48" s="13"/>
       <c r="J48" s="8"/>
-      <c r="K48" s="8"/>
-      <c r="L48" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="49" spans="2:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="K48" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="L48" s="8"/>
+    </row>
+    <row r="49" spans="2:12" ht="66" x14ac:dyDescent="0.3">
       <c r="B49" s="10"/>
-      <c r="C49" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D49" s="6">
-        <v>45625</v>
-      </c>
+      <c r="C49" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="8"/>
       <c r="E49" s="7" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="F49" s="8"/>
-      <c r="G49" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="I49" s="13"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="8"/>
       <c r="J49" s="8"/>
-      <c r="K49" s="5" t="s">
-        <v>60</v>
-      </c>
+      <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="2:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="B50" s="10"/>
-      <c r="C50" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D50" s="8"/>
+      <c r="C50" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50" s="6">
+        <v>45627</v>
+      </c>
       <c r="E50" s="7" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
-      <c r="J50" s="8"/>
-      <c r="K50" s="8"/>
+      <c r="J50" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K50" s="13"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
-      <c r="B51" s="10"/>
+    <row r="51" spans="2:12" ht="33" x14ac:dyDescent="0.3">
+      <c r="B51" s="4">
+        <v>15</v>
+      </c>
       <c r="C51" s="5" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="D51" s="6">
-        <v>45627</v>
+        <v>45630</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="8"/>
-      <c r="J51" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="K51" s="13"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
       <c r="L51" s="8"/>
     </row>
-    <row r="52" spans="2:12" ht="33" x14ac:dyDescent="0.3">
-      <c r="B52" s="4">
-        <v>15</v>
-      </c>
+    <row r="52" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="B52" s="10"/>
       <c r="C52" s="5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D52" s="6">
-        <v>45630</v>
+        <v>45632</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
@@ -2923,69 +2905,50 @@
       <c r="I52" s="8"/>
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
-      <c r="L52" s="8"/>
-    </row>
-    <row r="53" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="L52" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12" ht="66" x14ac:dyDescent="0.3">
       <c r="B53" s="10"/>
-      <c r="C53" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" s="6">
-        <v>45632</v>
-      </c>
+      <c r="C53" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="8"/>
       <c r="E53" s="7" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
       <c r="H53" s="8"/>
       <c r="I53" s="8"/>
-      <c r="J53" s="8"/>
-      <c r="K53" s="8"/>
-      <c r="L53" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="54" spans="2:12" ht="66" x14ac:dyDescent="0.3">
-      <c r="B54" s="10"/>
-      <c r="C54" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D54" s="8"/>
+      <c r="J53" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="K53" s="13"/>
+      <c r="L53" s="8"/>
+    </row>
+    <row r="54" spans="2:12" ht="165" x14ac:dyDescent="0.3">
+      <c r="B54" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C54" s="8"/>
+      <c r="D54" s="6">
+        <v>45639</v>
+      </c>
       <c r="E54" s="7" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
       <c r="J54" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="K54" s="13"/>
-      <c r="L54" s="8"/>
-    </row>
-    <row r="55" spans="2:12" ht="165" x14ac:dyDescent="0.3">
-      <c r="B55" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C55" s="8"/>
-      <c r="D55" s="6">
-        <v>45639</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="8"/>
-      <c r="I55" s="8"/>
-      <c r="J55" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="K55" s="8"/>
-      <c r="L55" s="5" t="s">
-        <v>72</v>
+        <v>59</v>
+      </c>
+      <c r="K54" s="8"/>
+      <c r="L54" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated schedule and added logistic comparison lecture and activity
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CFB1A67-2111-470D-88E9-BC0B17A3CC04}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C9DA52D-7ADE-41AD-A2EF-99325BF07591}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="195">
   <si>
     <t>week</t>
   </si>
@@ -603,9 +603,6 @@
     <t>/hw/hw-10.html</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Peer Review Due/HW 10 Due</t>
   </si>
   <si>
@@ -616,6 +613,12 @@
   </si>
   <si>
     <t>/project-instructions.html#peer-review</t>
+  </si>
+  <si>
+    <t>/slides/31-logistic-compare.html</t>
+  </si>
+  <si>
+    <t>/ae/ae-23-comparing-logistic.html</t>
   </si>
 </sst>
 </file>
@@ -2642,7 +2645,7 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -2654,19 +2657,23 @@
         <v>45616</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
+        <v>180</v>
+      </c>
+      <c r="G41" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>184</v>
+      </c>
       <c r="I41" s="8"/>
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="5"/>
     </row>
-    <row r="42" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -2678,11 +2685,17 @@
         <v>45618</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="F42" s="8"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="9"/>
+        <v>187</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="G42" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>194</v>
+      </c>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
@@ -2702,17 +2715,17 @@
         <v>45621</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="5"/>
       <c r="H43" s="9"/>
       <c r="I43" s="13"/>
       <c r="J43" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L43" s="8"/>
     </row>
@@ -2728,7 +2741,7 @@
         <v>45623</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>

</xml_diff>

<commit_message>
Fixed schedule link issue
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C9DA52D-7ADE-41AD-A2EF-99325BF07591}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F532335-3CB6-4F4B-8421-7C00ED355DF8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
@@ -615,10 +615,10 @@
     <t>/project-instructions.html#peer-review</t>
   </si>
   <si>
-    <t>/slides/31-logistic-compare.html</t>
-  </si>
-  <si>
-    <t>/ae/ae-23-comparing-logistic.html</t>
+    <t>/ae/ae-24-comparing-logistic.html</t>
+  </si>
+  <si>
+    <t>/slides/31-logistic-comparison.html</t>
   </si>
 </sst>
 </file>
@@ -1168,10 +1168,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2691,10 +2687,10 @@
         <v>185</v>
       </c>
       <c r="G42" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="H42" s="9" t="s">
         <v>193</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>194</v>
       </c>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>

</xml_diff>

<commit_message>
Added exam 2 review
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{B076A290-3229-49A8-82F8-02EAF0C6235B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F532335-3CB6-4F4B-8421-7C00ED355DF8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D3DD1A-D125-4A71-B600-FE483BAB3152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="197">
   <si>
     <t>week</t>
   </si>
@@ -619,13 +619,19 @@
   </si>
   <si>
     <t>/slides/31-logistic-comparison.html</t>
+  </si>
+  <si>
+    <t>/slides/32-exam02-review.html</t>
+  </si>
+  <si>
+    <t>/ae/exam-02-review.html</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1488,12 +1494,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C666FC1-734D-4F31-9D28-5509B94BC597}">
   <dimension ref="A1:L54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="16.5">
       <c r="A1" s="17" t="s">
         <v>61</v>
       </c>
@@ -1531,7 +1537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="49.5">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -1560,7 +1566,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="33">
       <c r="A3" t="s">
         <v>62</v>
       </c>
@@ -1587,7 +1593,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="66">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1611,7 +1617,7 @@
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
     </row>
-    <row r="5" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="66">
       <c r="A5" t="s">
         <v>62</v>
       </c>
@@ -1645,7 +1651,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="49.5">
       <c r="A6" t="s">
         <v>62</v>
       </c>
@@ -1671,7 +1677,7 @@
       <c r="K6" s="28"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16.5">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -1688,7 +1694,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="99">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1720,7 +1726,7 @@
       </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="181.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="165">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -1752,7 +1758,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="115.5">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -1780,7 +1786,7 @@
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="148.5">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -1805,7 +1811,7 @@
       <c r="K11" s="5"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="66">
       <c r="A12" t="s">
         <v>62</v>
       </c>
@@ -1837,7 +1843,7 @@
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="99">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -1867,7 +1873,7 @@
       <c r="K13" s="36"/>
       <c r="L13" s="35"/>
     </row>
-    <row r="14" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="66">
       <c r="A14" t="s">
         <v>62</v>
       </c>
@@ -1895,7 +1901,7 @@
       <c r="K14" s="36"/>
       <c r="L14" s="35"/>
     </row>
-    <row r="15" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="49.5">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -1927,7 +1933,7 @@
       </c>
       <c r="L15" s="35"/>
     </row>
-    <row r="16" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="49.5">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -1957,7 +1963,7 @@
       </c>
       <c r="L16" s="35"/>
     </row>
-    <row r="17" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="99">
       <c r="A17" t="s">
         <v>62</v>
       </c>
@@ -1976,7 +1982,7 @@
       <c r="K17" s="36"/>
       <c r="L17" s="35"/>
     </row>
-    <row r="18" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="33">
       <c r="A18" t="s">
         <v>62</v>
       </c>
@@ -2008,7 +2014,7 @@
       </c>
       <c r="L18" s="35"/>
     </row>
-    <row r="19" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="66">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -2037,7 +2043,7 @@
       <c r="J19" s="24"/>
       <c r="L19" s="24"/>
     </row>
-    <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="66">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -2065,7 +2071,7 @@
       <c r="K20" s="25"/>
       <c r="L20" s="25"/>
     </row>
-    <row r="21" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="49.5">
       <c r="A21" t="s">
         <v>62</v>
       </c>
@@ -2097,7 +2103,7 @@
       </c>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="66">
       <c r="A22" t="s">
         <v>62</v>
       </c>
@@ -2127,7 +2133,7 @@
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="33">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -2155,7 +2161,7 @@
       <c r="K23" s="5"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="16.5">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -2179,7 +2185,7 @@
       </c>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="66">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -2205,7 +2211,7 @@
       </c>
       <c r="L25" s="8"/>
     </row>
-    <row r="26" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="66">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -2227,7 +2233,7 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
     </row>
-    <row r="27" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="66">
       <c r="A27" t="s">
         <v>62</v>
       </c>
@@ -2249,7 +2255,7 @@
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="49.5">
       <c r="A28" t="s">
         <v>62</v>
       </c>
@@ -2279,7 +2285,7 @@
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="66">
       <c r="A29" t="s">
         <v>62</v>
       </c>
@@ -2309,7 +2315,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="99">
       <c r="A30" t="s">
         <v>62</v>
       </c>
@@ -2339,7 +2345,7 @@
       </c>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="49.5">
       <c r="A31" t="s">
         <v>62</v>
       </c>
@@ -2369,7 +2375,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="49.5">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -2401,7 +2407,7 @@
       </c>
       <c r="L32" s="48"/>
     </row>
-    <row r="33" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="82.5">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -2432,7 +2438,7 @@
       </c>
       <c r="L33" s="51"/>
     </row>
-    <row r="34" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="49.5">
       <c r="A34" t="s">
         <v>62</v>
       </c>
@@ -2462,7 +2468,7 @@
       <c r="K34" s="50"/>
       <c r="L34" s="49"/>
     </row>
-    <row r="35" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" ht="82.5">
       <c r="A35" t="s">
         <v>62</v>
       </c>
@@ -2490,7 +2496,7 @@
       <c r="K35" s="13"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="82.5">
       <c r="A36" t="s">
         <v>62</v>
       </c>
@@ -2519,7 +2525,7 @@
       </c>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="82.5">
       <c r="A37" t="s">
         <v>62</v>
       </c>
@@ -2547,7 +2553,7 @@
       <c r="K37" s="5"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" ht="82.5">
       <c r="A38" t="s">
         <v>62</v>
       </c>
@@ -2575,7 +2581,7 @@
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="115.5">
       <c r="A39" t="s">
         <v>62</v>
       </c>
@@ -2605,7 +2611,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" ht="66">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -2641,7 +2647,7 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="66">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -2669,7 +2675,7 @@
       <c r="K41" s="8"/>
       <c r="L41" s="5"/>
     </row>
-    <row r="42" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="99">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -2697,7 +2703,7 @@
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="33">
       <c r="A43" t="s">
         <v>62</v>
       </c>
@@ -2714,8 +2720,12 @@
         <v>190</v>
       </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="9"/>
+      <c r="G43" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>196</v>
+      </c>
       <c r="I43" s="13"/>
       <c r="J43" s="8" t="s">
         <v>192</v>
@@ -2725,7 +2735,7 @@
       </c>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="16.5">
       <c r="A44" t="s">
         <v>62</v>
       </c>
@@ -2747,7 +2757,7 @@
       <c r="K44" s="13"/>
       <c r="L44" s="12"/>
     </row>
-    <row r="45" spans="1:12" ht="86.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="86.25" customHeight="1">
       <c r="A45" t="s">
         <v>62</v>
       </c>
@@ -2769,7 +2779,7 @@
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="66">
       <c r="B46" s="10"/>
       <c r="C46" s="9" t="s">
         <v>18</v>
@@ -2786,7 +2796,7 @@
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" ht="148.5">
       <c r="B47" s="4">
         <v>14</v>
       </c>
@@ -2813,7 +2823,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" ht="33">
       <c r="B48" s="10"/>
       <c r="C48" s="5" t="s">
         <v>11</v>
@@ -2838,7 +2848,7 @@
       </c>
       <c r="L48" s="8"/>
     </row>
-    <row r="49" spans="2:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:12" ht="49.5">
       <c r="B49" s="10"/>
       <c r="C49" s="9" t="s">
         <v>18</v>
@@ -2855,7 +2865,7 @@
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:12" ht="82.5">
       <c r="B50" s="10"/>
       <c r="C50" s="5" t="s">
         <v>49</v>
@@ -2876,7 +2886,7 @@
       <c r="K50" s="13"/>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="2:12" ht="33" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:12" ht="16.5">
       <c r="B51" s="4">
         <v>15</v>
       </c>
@@ -2897,7 +2907,7 @@
       <c r="K51" s="8"/>
       <c r="L51" s="8"/>
     </row>
-    <row r="52" spans="2:12" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:12" ht="99">
       <c r="B52" s="10"/>
       <c r="C52" s="5" t="s">
         <v>11</v>
@@ -2918,7 +2928,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="53" spans="2:12" ht="66" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:12" ht="66">
       <c r="B53" s="10"/>
       <c r="C53" s="9" t="s">
         <v>18</v>
@@ -2937,7 +2947,7 @@
       <c r="K53" s="13"/>
       <c r="L53" s="8"/>
     </row>
-    <row r="54" spans="2:12" ht="165" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:12" ht="115.5">
       <c r="B54" s="4" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Updating schedule and final lecture
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Dropbox\OneDrive - The College of Idaho\Teaching\MAT212FA24\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yotescollegeofidaho-my.sharepoint.com/personal/efriedlander_collegeofidaho_edu/Documents/Teaching/MAT212FA24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFFA4DE-32A9-420F-A62C-6196583D259C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{7CFFA4DE-32A9-420F-A62C-6196583D259C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41D97806-E176-4EE9-9FFD-E02E89FBA51E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82B2C154-7672-424B-83B7-3BF61C3BA031}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="187">
   <si>
     <t>week</t>
   </si>
@@ -90,9 +90,6 @@
     <t>/slides/02-big-picture.html</t>
   </si>
   <si>
-    <t>Tu &amp; Th</t>
-  </si>
-  <si>
     <t>M</t>
   </si>
   <si>
@@ -144,9 +141,6 @@
     <t>/hw/hw-04.html</t>
   </si>
   <si>
-    <t>Lab: Work on project</t>
-  </si>
-  <si>
     <t>Logistic regression: Inference</t>
   </si>
   <si>
@@ -156,69 +150,9 @@
     <t>NO LECTURE: Thanksgiving Break</t>
   </si>
   <si>
-    <t>NO LAB: Thanksgiving Break</t>
-  </si>
-  <si>
-    <t>Multinomial logistic regression: Prediction + Inference</t>
-  </si>
-  <si>
-    <t>/prepare/nov-27.html</t>
-  </si>
-  <si>
-    <t>/slides/22-multinomial-logistic-pt2.html</t>
-  </si>
-  <si>
-    <t>Project work day?</t>
-  </si>
-  <si>
-    <t>Exam 02 Review</t>
-  </si>
-  <si>
-    <t>/slides/23-exam-02-review.html</t>
-  </si>
-  <si>
-    <t>/ae/ae-17-exam-02-review.html</t>
-  </si>
-  <si>
-    <t>HW 05 due</t>
-  </si>
-  <si>
-    <t>Fr</t>
-  </si>
-  <si>
-    <t>Round 1 submission due (optional)</t>
-  </si>
-  <si>
-    <t>/project-instructions.html#round1-submission</t>
-  </si>
-  <si>
-    <t>Exam 02</t>
-  </si>
-  <si>
-    <t>No Lecture: Work on Exam 02 take-home</t>
-  </si>
-  <si>
     <t>Something related to statistics experience/ alumni?</t>
   </si>
   <si>
-    <t>Lab: Project presentations</t>
-  </si>
-  <si>
-    <t>https://sta210-fa23.netlify.app/project-instructions#presentation</t>
-  </si>
-  <si>
-    <t>Exam period</t>
-  </si>
-  <si>
-    <t>Project: Final written report + Organized GitHub repo due</t>
-  </si>
-  <si>
-    <t>https://sta210-fa23.netlify.app/project-instructions#written-report</t>
-  </si>
-  <si>
-    <t>Reading period 12/9 - 12/12 (don’t have anything due)</t>
-  </si>
-  <si>
     <t>Publish</t>
   </si>
   <si>
@@ -625,13 +559,49 @@
   </si>
   <si>
     <t>/slides/32-exam-02-review.html</t>
+  </si>
+  <si>
+    <t>Work on Project</t>
+  </si>
+  <si>
+    <t>Final Paper Due</t>
+  </si>
+  <si>
+    <t>https://cofi.instructure.com/courses/15692/assignments/201717</t>
+  </si>
+  <si>
+    <t>Exam Corrections Due</t>
+  </si>
+  <si>
+    <t>/project-instructions#written-report.html</t>
+  </si>
+  <si>
+    <t>Finals Week</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Final Poster Due</t>
+  </si>
+  <si>
+    <t>/project-instructions#poster-presentation.html</t>
+  </si>
+  <si>
+    <t>Final Poster Due in Canvas</t>
+  </si>
+  <si>
+    <t>Final Poster Presentation: CML 105 8:30am - 11am</t>
+  </si>
+  <si>
+    <t>Final Poster Presentation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1003,7 +973,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -1048,9 +1018,6 @@
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
@@ -1493,15 +1460,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C666FC1-734D-4F31-9D28-5509B94BC597}">
-  <dimension ref="A1:L54"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:L51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5">
-      <c r="A1" s="17" t="s">
-        <v>61</v>
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1537,9 +1504,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="49.5">
+    <row r="2" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
@@ -1557,18 +1524,18 @@
       <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="18" t="s">
-        <v>64</v>
+      <c r="I2" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
       <c r="L2" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="33">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="5" t="s">
@@ -1581,7 +1548,7 @@
         <v>16</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
@@ -1590,36 +1557,36 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="L3" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="66">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" s="6">
         <v>45530</v>
       </c>
-      <c r="E4" s="19" t="s">
-        <v>67</v>
+      <c r="E4" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
     </row>
-    <row r="5" spans="1:12" ht="66">
+    <row r="5" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="5" t="s">
@@ -1629,31 +1596,31 @@
         <v>45532</v>
       </c>
       <c r="E5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>21</v>
-      </c>
       <c r="G5" s="5" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="18" t="s">
-        <v>25</v>
+      <c r="I5" s="17" t="s">
+        <v>24</v>
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="49.5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="5" t="s">
@@ -1663,40 +1630,40 @@
         <v>45534</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
-      <c r="K6" s="28"/>
+      <c r="K6" s="27"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="16.5">
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B7" s="4">
         <v>3</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="6">
         <v>45537</v>
       </c>
-      <c r="E7" s="29" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="99">
+      <c r="E7" s="28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5" t="s">
@@ -1706,29 +1673,29 @@
         <v>45539</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>75</v>
+        <v>22</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>53</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:12" ht="165">
+    <row r="9" spans="1:12" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="5" t="s">
@@ -1738,47 +1705,47 @@
         <v>45541</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="8"/>
       <c r="K9" s="9" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="115.5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B10" s="4">
         <v>4</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" s="6">
         <v>45544</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="8"/>
@@ -1786,9 +1753,9 @@
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" ht="148.5">
+    <row r="11" spans="1:12" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="5" t="s">
@@ -1798,22 +1765,22 @@
         <v>45546</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="5" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="5"/>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" ht="66">
+    <row r="12" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="5" t="s">
@@ -1823,319 +1790,319 @@
         <v>45548</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="31" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="I12" s="30" t="s">
+        <v>31</v>
       </c>
       <c r="J12" s="8"/>
       <c r="K12" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="L12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" ht="99" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="31">
+        <v>5</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="33">
+        <v>45551</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13" s="36"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="34"/>
+    </row>
+    <row r="14" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="33">
+        <v>45553</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" s="36"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="34"/>
+    </row>
+    <row r="15" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="31"/>
+      <c r="C15" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="33">
+        <v>45555</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="I15" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J15" s="34"/>
+      <c r="K15" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="L15" s="34"/>
+    </row>
+    <row r="16" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="31">
+        <v>6</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="33">
+        <v>45558</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="G16" s="35"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="36"/>
+      <c r="J16" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="K16" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="L16" s="34"/>
+    </row>
+    <row r="17" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="31"/>
+      <c r="C17" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="33">
+        <v>45560</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="L12" s="8"/>
-    </row>
-    <row r="13" spans="1:12" ht="99">
-      <c r="A13" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="32">
-        <v>5</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="34">
-        <v>45551</v>
-      </c>
-      <c r="E13" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="I13" s="37"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36"/>
-      <c r="L13" s="35"/>
-    </row>
-    <row r="14" spans="1:12" ht="66">
-      <c r="A14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="34">
-        <v>45553</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="35"/>
-    </row>
-    <row r="15" spans="1:12" ht="49.5">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="33" t="s">
+      <c r="I17" s="36"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="34"/>
+    </row>
+    <row r="18" spans="1:12" ht="33" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="34">
-        <v>45555</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="F15" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="G15" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="H15" s="39" t="s">
-        <v>104</v>
-      </c>
-      <c r="I15" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="L15" s="35"/>
-    </row>
-    <row r="16" spans="1:12" ht="49.5">
-      <c r="A16" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="32">
-        <v>6</v>
-      </c>
-      <c r="C16" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="34">
-        <v>45558</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>108</v>
-      </c>
-      <c r="G16" s="36"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="52" t="s">
-        <v>33</v>
-      </c>
-      <c r="K16" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="L16" s="35"/>
-    </row>
-    <row r="17" spans="1:12" ht="99">
-      <c r="A17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="34">
-        <v>45560</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="I17" s="37"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="35"/>
-    </row>
-    <row r="18" spans="1:12" ht="33">
-      <c r="A18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="34">
+      <c r="D18" s="33">
         <v>45562</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="G18" s="36" t="s">
-        <v>103</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>106</v>
-      </c>
-      <c r="I18" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="J18" s="35"/>
-      <c r="K18" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="L18" s="35"/>
-    </row>
-    <row r="19" spans="1:12" ht="66">
+        <v>77</v>
+      </c>
+      <c r="F18" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" s="35" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="J18" s="34"/>
+      <c r="K18" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="L18" s="34"/>
+    </row>
+    <row r="19" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B19" s="4">
         <v>7</v>
       </c>
-      <c r="C19" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="22">
+      <c r="C19" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="21">
         <v>45565</v>
       </c>
       <c r="E19" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="L19" s="23"/>
+    </row>
+    <row r="20" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="22">
+        <v>45567</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+    </row>
+    <row r="21" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="22">
+        <v>45569</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="H19" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="L19" s="24"/>
-    </row>
-    <row r="20" spans="1:12" ht="66">
-      <c r="A20" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="42" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="23">
-        <v>45567</v>
-      </c>
-      <c r="E20" s="40" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="G20" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="H20" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-    </row>
-    <row r="21" spans="1:12" ht="49.5">
-      <c r="A21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="23">
-        <v>45569</v>
-      </c>
-      <c r="E21" s="43" t="s">
-        <v>114</v>
-      </c>
-      <c r="F21" s="45" t="s">
-        <v>128</v>
-      </c>
-      <c r="G21" s="26" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>120</v>
+      <c r="H21" s="26" t="s">
+        <v>98</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="8" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="L21" s="8"/>
     </row>
-    <row r="22" spans="1:12" ht="66">
+    <row r="22" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B22" s="4">
         <v>8</v>
       </c>
-      <c r="C22" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="47">
+      <c r="C22" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="46">
         <v>45572</v>
       </c>
-      <c r="E22" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="F22" s="45" t="s">
-        <v>127</v>
-      </c>
-      <c r="G22" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>130</v>
+      <c r="E22" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="G22" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="H22" s="26" t="s">
+        <v>108</v>
       </c>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
-    <row r="23" spans="1:12" ht="33">
+    <row r="23" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="5" t="s">
@@ -2145,25 +2112,25 @@
         <v>45574</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="G23" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>131</v>
+        <v>29</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="H23" s="26" t="s">
+        <v>109</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
       <c r="K23" s="5"/>
       <c r="L23" s="8"/>
     </row>
-    <row r="24" spans="1:12" ht="16.5">
+    <row r="24" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="5" t="s">
@@ -2173,7 +2140,7 @@
         <v>45576</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
@@ -2181,25 +2148,25 @@
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="L24" s="8"/>
     </row>
-    <row r="25" spans="1:12" ht="66">
+    <row r="25" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B25" s="4">
         <v>9</v>
       </c>
-      <c r="C25" s="38" t="s">
-        <v>19</v>
+      <c r="C25" s="37" t="s">
+        <v>18</v>
       </c>
       <c r="D25" s="6">
         <v>45579</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -2207,13 +2174,13 @@
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="L25" s="8"/>
     </row>
-    <row r="26" spans="1:12" ht="66">
+    <row r="26" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="9" t="s">
@@ -2223,7 +2190,7 @@
         <v>45581</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -2233,9 +2200,9 @@
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
     </row>
-    <row r="27" spans="1:12" ht="66">
+    <row r="27" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="5" t="s">
@@ -2245,7 +2212,7 @@
         <v>45583</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
@@ -2255,39 +2222,39 @@
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:12" ht="49.5">
+    <row r="28" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B28" s="4">
         <v>10</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D28" s="6">
         <v>45586</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="G28" s="26" t="s">
-        <v>134</v>
+        <v>106</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>112</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="I28" s="13"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
     </row>
-    <row r="29" spans="1:12" ht="66">
+    <row r="29" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="9" t="s">
@@ -2297,27 +2264,27 @@
         <v>45588</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="G29" s="26" t="s">
-        <v>137</v>
+        <v>117</v>
+      </c>
+      <c r="G29" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
       <c r="L29" s="5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="99">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="5" t="s">
@@ -2327,57 +2294,57 @@
         <v>45590</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="F30" s="8"/>
-      <c r="G30" s="26" t="s">
-        <v>141</v>
+      <c r="G30" s="25" t="s">
+        <v>119</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="L30" s="8"/>
     </row>
-    <row r="31" spans="1:12" ht="49.5">
+    <row r="31" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B31" s="4">
         <v>11</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D31" s="6">
         <v>45593</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>151</v>
+        <v>128</v>
+      </c>
+      <c r="G31" s="25" t="s">
+        <v>129</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>152</v>
+        <v>130</v>
       </c>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
     </row>
-    <row r="32" spans="1:12" ht="49.5">
+    <row r="32" spans="1:12" ht="66" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="9" t="s">
@@ -2387,29 +2354,29 @@
         <v>45595</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="G32" s="26" t="s">
-        <v>155</v>
+        <v>131</v>
+      </c>
+      <c r="G32" s="25" t="s">
+        <v>133</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="I32" s="48"/>
-      <c r="J32" s="51" t="s">
-        <v>145</v>
-      </c>
-      <c r="K32" s="48" t="s">
-        <v>146</v>
-      </c>
-      <c r="L32" s="48"/>
-    </row>
-    <row r="33" spans="1:12" ht="82.5">
+        <v>134</v>
+      </c>
+      <c r="I32" s="47"/>
+      <c r="J32" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="K32" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="L32" s="47"/>
+    </row>
+    <row r="33" spans="1:12" ht="99" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="5" t="s">
@@ -2419,58 +2386,58 @@
         <v>45597</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>155</v>
+        <v>131</v>
+      </c>
+      <c r="G33" s="25" t="s">
+        <v>133</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>156</v>
+        <v>134</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="K33" s="51" t="s">
-        <v>144</v>
-      </c>
-      <c r="L33" s="51"/>
-    </row>
-    <row r="34" spans="1:12" ht="49.5">
+        <v>139</v>
+      </c>
+      <c r="K33" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="L33" s="50"/>
+    </row>
+    <row r="34" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B34" s="4">
         <v>12</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D34" s="6">
         <v>45600</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>158</v>
+        <v>135</v>
+      </c>
+      <c r="G34" s="25" t="s">
+        <v>136</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="I34" s="50"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="50"/>
-      <c r="L34" s="49"/>
-    </row>
-    <row r="35" spans="1:12" ht="82.5">
+        <v>137</v>
+      </c>
+      <c r="I34" s="49"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="49"/>
+      <c r="L34" s="48"/>
+    </row>
+    <row r="35" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="9" t="s">
@@ -2480,25 +2447,25 @@
         <v>45602</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G35" s="26" t="s">
-        <v>164</v>
+        <v>135</v>
+      </c>
+      <c r="G35" s="25" t="s">
+        <v>142</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="I35" s="8"/>
       <c r="J35" s="9"/>
       <c r="K35" s="13"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="1:12" ht="82.5">
+    <row r="36" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="5" t="s">
@@ -2508,44 +2475,44 @@
         <v>45604</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="G36" s="26" t="s">
-        <v>171</v>
+        <v>148</v>
+      </c>
+      <c r="G36" s="25" t="s">
+        <v>149</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>167</v>
+        <v>145</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="J36" s="8"/>
-      <c r="K36" s="51" t="s">
-        <v>163</v>
+      <c r="K36" s="50" t="s">
+        <v>141</v>
       </c>
       <c r="L36" s="8"/>
     </row>
-    <row r="37" spans="1:12" ht="82.5">
+    <row r="37" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B37" s="4">
         <v>13</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D37" s="6">
         <v>45607</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="G37" s="26" t="s">
-        <v>182</v>
+        <v>144</v>
+      </c>
+      <c r="G37" s="25" t="s">
+        <v>160</v>
       </c>
       <c r="H37" s="9"/>
       <c r="I37" s="8"/>
@@ -2553,9 +2520,9 @@
       <c r="K37" s="5"/>
       <c r="L37" s="8"/>
     </row>
-    <row r="38" spans="1:12" ht="82.5">
+    <row r="38" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="5" t="s">
@@ -2565,25 +2532,25 @@
         <v>45609</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="G38" s="26" t="s">
-        <v>174</v>
+        <v>147</v>
+      </c>
+      <c r="G38" s="25" t="s">
+        <v>152</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="I38" s="8"/>
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" ht="115.5">
+    <row r="39" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="5" t="s">
@@ -2593,63 +2560,63 @@
         <v>45611</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="G39" s="26" t="s">
-        <v>175</v>
+        <v>147</v>
+      </c>
+      <c r="G39" s="25" t="s">
+        <v>153</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="I39" s="8"/>
       <c r="J39" s="8"/>
       <c r="K39" s="8" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" ht="66">
+    <row r="40" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B40" s="4">
         <v>14</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D40" s="6">
         <v>45614</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="G40" s="26" t="s">
-        <v>183</v>
+        <v>158</v>
+      </c>
+      <c r="G40" s="25" t="s">
+        <v>161</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>188</v>
+        <v>166</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>186</v>
+        <v>164</v>
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" ht="66">
+    <row r="41" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B41" s="10"/>
       <c r="C41" s="9" t="s">
@@ -2659,25 +2626,25 @@
         <v>45616</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="G41" s="26" t="s">
-        <v>183</v>
+        <v>158</v>
+      </c>
+      <c r="G41" s="25" t="s">
+        <v>161</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="I41" s="8"/>
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="5"/>
     </row>
-    <row r="42" spans="1:12" ht="99">
+    <row r="42" spans="1:12" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="5" t="s">
@@ -2687,57 +2654,57 @@
         <v>45618</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="G42" s="26" t="s">
-        <v>194</v>
+        <v>158</v>
+      </c>
+      <c r="G42" s="25" t="s">
+        <v>161</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="I42" s="13"/>
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
     </row>
-    <row r="43" spans="1:12" ht="33">
+    <row r="43" spans="1:12" ht="33" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B43" s="4">
         <v>15</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D43" s="6">
         <v>45621</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="F43" s="8"/>
-      <c r="G43" s="26" t="s">
-        <v>196</v>
+      <c r="G43" s="25" t="s">
+        <v>174</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>195</v>
+        <v>173</v>
       </c>
       <c r="I43" s="13"/>
       <c r="J43" s="8" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>189</v>
+        <v>167</v>
       </c>
       <c r="L43" s="8"/>
     </row>
-    <row r="44" spans="1:12" ht="16.5">
+    <row r="44" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B44" s="10"/>
       <c r="C44" s="9" t="s">
@@ -2747,7 +2714,7 @@
         <v>45623</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>191</v>
+        <v>169</v>
       </c>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
@@ -2757,9 +2724,9 @@
       <c r="K44" s="13"/>
       <c r="L44" s="12"/>
     </row>
-    <row r="45" spans="1:12" ht="86.25" customHeight="1">
+    <row r="45" spans="1:12" ht="86.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="B45" s="10"/>
       <c r="C45" s="5" t="s">
@@ -2769,7 +2736,7 @@
         <v>45625</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
@@ -2779,195 +2746,163 @@
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" ht="66">
-      <c r="B46" s="10"/>
-      <c r="C46" s="9" t="s">
+    <row r="46" spans="1:12" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="4">
+        <v>16</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D46" s="8"/>
-      <c r="E46" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
+      <c r="D46" s="6">
+        <v>45628</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="G46" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="H46" s="9" t="s">
+        <v>171</v>
+      </c>
       <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
       <c r="K46" s="8"/>
-      <c r="L46" s="8"/>
-    </row>
-    <row r="47" spans="1:12" ht="148.5">
-      <c r="B47" s="4">
-        <v>14</v>
-      </c>
+      <c r="L46" s="5"/>
+    </row>
+    <row r="47" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47" s="10"/>
       <c r="C47" s="5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D47" s="6">
-        <v>45623</v>
+        <v>45630</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H47" s="13"/>
-      <c r="I47" s="8"/>
+        <v>175</v>
+      </c>
+      <c r="F47" s="8"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="13"/>
       <c r="J47" s="8"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" ht="33">
+      <c r="K47" s="5"/>
+      <c r="L47" s="8"/>
+    </row>
+    <row r="48" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>40</v>
+      </c>
       <c r="B48" s="10"/>
-      <c r="C48" s="5" t="s">
-        <v>11</v>
+      <c r="C48" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="D48" s="6">
-        <v>45625</v>
+        <v>45632</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>45</v>
+        <v>175</v>
       </c>
       <c r="F48" s="8"/>
-      <c r="G48" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H48" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="I48" s="13"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="8" t="s">
+        <v>177</v>
+      </c>
       <c r="J48" s="8"/>
-      <c r="K48" s="5" t="s">
-        <v>48</v>
+      <c r="K48" s="8" t="s">
+        <v>178</v>
       </c>
       <c r="L48" s="8"/>
     </row>
-    <row r="49" spans="2:12" ht="49.5">
-      <c r="B49" s="10"/>
-      <c r="C49" s="9" t="s">
+    <row r="49" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="8"/>
+      <c r="D49" s="6">
+        <v>45635</v>
+      </c>
       <c r="E49" s="7" t="s">
-        <v>36</v>
+        <v>176</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
       <c r="I49" s="8"/>
-      <c r="J49" s="8"/>
-      <c r="K49" s="8"/>
+      <c r="J49" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="K49" s="13" t="s">
+        <v>176</v>
+      </c>
       <c r="L49" s="8"/>
     </row>
-    <row r="50" spans="2:12" ht="82.5">
-      <c r="B50" s="10"/>
+    <row r="50" spans="1:12" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" s="4"/>
       <c r="C50" s="5" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
       <c r="D50" s="6">
-        <v>45627</v>
+        <v>45636</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>50</v>
+        <v>182</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
-      <c r="J50" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K50" s="13"/>
+      <c r="J50" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="K50" s="8" t="s">
+        <v>184</v>
+      </c>
       <c r="L50" s="8"/>
     </row>
-    <row r="51" spans="2:12" ht="16.5">
-      <c r="B51" s="4">
-        <v>15</v>
-      </c>
+    <row r="51" spans="1:12" ht="66" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>40</v>
+      </c>
+      <c r="B51" s="10"/>
       <c r="C51" s="5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D51" s="6">
-        <v>45630</v>
+        <v>45637</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>52</v>
+        <v>186</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="8"/>
-      <c r="J51" s="8"/>
-      <c r="K51" s="8"/>
-      <c r="L51" s="8"/>
-    </row>
-    <row r="52" spans="2:12" ht="99">
-      <c r="B52" s="10"/>
-      <c r="C52" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" s="6">
-        <v>45632</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F52" s="8"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="8"/>
-      <c r="I52" s="8"/>
-      <c r="J52" s="8"/>
-      <c r="K52" s="8"/>
-      <c r="L52" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="53" spans="2:12" ht="66">
-      <c r="B53" s="10"/>
-      <c r="C53" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D53" s="8"/>
-      <c r="E53" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="8"/>
-      <c r="J53" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="K53" s="13"/>
-      <c r="L53" s="8"/>
-    </row>
-    <row r="54" spans="2:12" ht="115.5">
-      <c r="B54" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="8"/>
-      <c r="D54" s="6">
-        <v>45639</v>
-      </c>
-      <c r="E54" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="K54" s="8"/>
-      <c r="L54" s="5" t="s">
-        <v>60</v>
+      <c r="J51" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="K51" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="L51" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>